<commit_message>
fixed staff report bug & workorder export report bug
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/wo/woExport/APM_WorkOrder_Template.xlsx
+++ b/src/src/main/webapp/portal/wo/woExport/APM_WorkOrder_Template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>报修单号</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -135,6 +135,10 @@
   </si>
   <si>
     <t>验收人</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>资产编号</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -483,32 +487,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="20.5" customWidth="1"/>
-    <col min="3" max="3" width="23.125" customWidth="1"/>
-    <col min="4" max="4" width="16.375" customWidth="1"/>
-    <col min="5" max="5" width="17.5" customWidth="1"/>
-    <col min="6" max="6" width="20.375" customWidth="1"/>
-    <col min="7" max="7" width="16.25" customWidth="1"/>
-    <col min="8" max="8" width="15.875" customWidth="1"/>
-    <col min="9" max="9" width="25.375" customWidth="1"/>
-    <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.125" customWidth="1"/>
-    <col min="12" max="12" width="14.625" customWidth="1"/>
-    <col min="13" max="13" width="26.125" customWidth="1"/>
-    <col min="14" max="14" width="25" customWidth="1"/>
-    <col min="15" max="15" width="16.375" customWidth="1"/>
-    <col min="16" max="16" width="12.25" customWidth="1"/>
-    <col min="17" max="17" width="25" customWidth="1"/>
-    <col min="20" max="20" width="23.625" customWidth="1"/>
-    <col min="21" max="22" width="25.875" customWidth="1"/>
-    <col min="23" max="23" width="17" customWidth="1"/>
-    <col min="24" max="24" width="16.125" customWidth="1"/>
+    <col min="2" max="3" width="20.5" customWidth="1"/>
+    <col min="4" max="4" width="23.125" customWidth="1"/>
+    <col min="5" max="5" width="16.375" customWidth="1"/>
+    <col min="6" max="6" width="17.5" customWidth="1"/>
+    <col min="7" max="7" width="20.375" customWidth="1"/>
+    <col min="8" max="8" width="16.25" customWidth="1"/>
+    <col min="9" max="9" width="15.875" customWidth="1"/>
+    <col min="10" max="10" width="25.375" customWidth="1"/>
+    <col min="11" max="11" width="23" customWidth="1"/>
+    <col min="12" max="12" width="14.125" customWidth="1"/>
+    <col min="13" max="13" width="14.625" customWidth="1"/>
+    <col min="14" max="14" width="26.125" customWidth="1"/>
+    <col min="15" max="15" width="25" customWidth="1"/>
+    <col min="16" max="16" width="16.375" customWidth="1"/>
+    <col min="17" max="17" width="12.25" customWidth="1"/>
+    <col min="18" max="18" width="25" customWidth="1"/>
+    <col min="21" max="21" width="23.625" customWidth="1"/>
+    <col min="22" max="23" width="25.875" customWidth="1"/>
+    <col min="24" max="24" width="17" customWidth="1"/>
+    <col min="25" max="25" width="16.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="16.5">
+    <row r="1" spans="1:25" ht="16.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -516,74 +520,77 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
-      <c r="Q2" s="2"/>
+    <row r="2" spans="1:25">
+      <c r="R2" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
add woreport export idea
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/wo/woExport/APM_WorkOrder_Template.xlsx
+++ b/src/src/main/webapp/portal/wo/woExport/APM_WorkOrder_Template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>报修单号</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -110,10 +110,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>价格</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>验收时间</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -143,6 +139,42 @@
   </si>
   <si>
     <t>工单状态</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>当前责任人</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>备注</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>当前步骤</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>解决方案</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>测试方法</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>问题描述</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>维修总费用</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>备件总费用</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>其他费用</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -491,32 +523,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="3" width="20.5" customWidth="1"/>
     <col min="4" max="5" width="23.125" customWidth="1"/>
     <col min="6" max="6" width="16.375" customWidth="1"/>
-    <col min="7" max="7" width="17.5" customWidth="1"/>
-    <col min="8" max="8" width="20.375" customWidth="1"/>
-    <col min="9" max="9" width="16.25" customWidth="1"/>
-    <col min="10" max="10" width="15.875" customWidth="1"/>
-    <col min="11" max="11" width="25.375" customWidth="1"/>
-    <col min="12" max="12" width="23" customWidth="1"/>
-    <col min="13" max="13" width="14.125" customWidth="1"/>
-    <col min="14" max="14" width="14.625" customWidth="1"/>
-    <col min="15" max="15" width="26.125" customWidth="1"/>
-    <col min="16" max="16" width="25" customWidth="1"/>
-    <col min="17" max="17" width="16.375" customWidth="1"/>
-    <col min="18" max="18" width="12.25" customWidth="1"/>
-    <col min="19" max="19" width="25" customWidth="1"/>
-    <col min="22" max="22" width="23.625" customWidth="1"/>
-    <col min="23" max="24" width="25.875" customWidth="1"/>
-    <col min="25" max="25" width="17" customWidth="1"/>
-    <col min="26" max="26" width="16.125" customWidth="1"/>
+    <col min="7" max="9" width="17.5" customWidth="1"/>
+    <col min="10" max="10" width="20.375" customWidth="1"/>
+    <col min="11" max="11" width="16.25" customWidth="1"/>
+    <col min="12" max="12" width="15.875" customWidth="1"/>
+    <col min="13" max="13" width="25.375" customWidth="1"/>
+    <col min="14" max="14" width="23" customWidth="1"/>
+    <col min="15" max="15" width="14.125" customWidth="1"/>
+    <col min="16" max="16" width="14.625" customWidth="1"/>
+    <col min="17" max="17" width="26.125" customWidth="1"/>
+    <col min="18" max="18" width="25" customWidth="1"/>
+    <col min="19" max="19" width="16.375" customWidth="1"/>
+    <col min="20" max="20" width="12.25" customWidth="1"/>
+    <col min="21" max="21" width="25" customWidth="1"/>
+    <col min="22" max="22" width="12.5" customWidth="1"/>
+    <col min="23" max="23" width="10.625" customWidth="1"/>
+    <col min="24" max="24" width="12.125" customWidth="1"/>
+    <col min="26" max="26" width="23.625" customWidth="1"/>
+    <col min="27" max="28" width="25.875" customWidth="1"/>
+    <col min="29" max="29" width="17" customWidth="1"/>
+    <col min="30" max="31" width="16.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="16.5">
+    <row r="1" spans="1:34" ht="16.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -524,13 +559,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -539,65 +574,91 @@
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="V1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="Z1" s="1" t="s">
-        <v>22</v>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:26">
-      <c r="S2" s="2"/>
+    <row r="2" spans="1:34">
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
add export ConfirmedDownTime and ConfirmedUpTime
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/wo/woExport/APM_WorkOrder_Template.xlsx
+++ b/src/src/main/webapp/portal/wo/woExport/APM_WorkOrder_Template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>报修单号</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -227,6 +227,14 @@
   </si>
   <si>
     <t>距上次报修天数</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>停机时间</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>恢复时间</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -575,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AU2"/>
+  <dimension ref="A1:AW2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="20.5" customWidth="1"/>
@@ -600,13 +608,13 @@
     <col min="36" max="36" width="23.625" customWidth="1"/>
     <col min="37" max="38" width="25.875" customWidth="1"/>
     <col min="39" max="39" width="21" customWidth="1"/>
-    <col min="40" max="40" width="25.875" customWidth="1"/>
-    <col min="41" max="41" width="16.25" customWidth="1"/>
-    <col min="42" max="42" width="17" customWidth="1"/>
-    <col min="43" max="44" width="16.125" customWidth="1"/>
+    <col min="40" max="42" width="25.875" customWidth="1"/>
+    <col min="43" max="43" width="16.25" customWidth="1"/>
+    <col min="44" max="44" width="17" customWidth="1"/>
+    <col min="45" max="46" width="16.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:49" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -728,28 +736,34 @@
         <v>36</v>
       </c>
       <c r="AO1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.2">
       <c r="AD2" s="2"/>
       <c r="AE2" s="2"/>
       <c r="AF2" s="2"/>

</xml_diff>